<commit_message>
2.6.2 Asignar tiempo para generar una solicitud - actualización de plantillas
</commit_message>
<xml_diff>
--- a/static/plantillas/BID-PMC-FOR-00017_Formato_de_Solicitud_de_Pruebas.xlsx
+++ b/static/plantillas/BID-PMC-FOR-00017_Formato_de_Solicitud_de_Pruebas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr showInkAnnotation="0" codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BID-eduardo.hernande\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BID-eduardo.hernande\Desktop\extractor\excel_extractor\static\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5DBB08D4-948A-416B-9386-6C671D86EAC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03476E57-3EDA-4D94-B62A-3DD9A9EEE9FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{174D9EE4-28BD-4DE1-BF18-35170CA27939}"/>
   </bookViews>
@@ -1458,6 +1458,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -1606,7 +1607,6 @@
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -3610,21 +3610,21 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B3" s="45" t="s">
+      <c r="B3" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="45"/>
-      <c r="I3" s="45"/>
-      <c r="J3" s="45"/>
-      <c r="K3" s="45"/>
-      <c r="L3" s="45"/>
-      <c r="M3" s="45"/>
-      <c r="N3" s="45"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
+      <c r="H3" s="46"/>
+      <c r="I3" s="46"/>
+      <c r="J3" s="46"/>
+      <c r="K3" s="46"/>
+      <c r="L3" s="46"/>
+      <c r="M3" s="46"/>
+      <c r="N3" s="46"/>
     </row>
     <row r="5" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="4" t="s">
@@ -3633,19 +3633,19 @@
       <c r="C5" s="2">
         <v>13</v>
       </c>
-      <c r="F5" s="46" t="s">
+      <c r="F5" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="G5" s="46"/>
+      <c r="G5" s="47"/>
       <c r="H5" s="2">
         <v>28</v>
       </c>
-      <c r="K5" s="45" t="s">
+      <c r="K5" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="L5" s="45"/>
-      <c r="M5" s="47"/>
-      <c r="N5" s="47"/>
+      <c r="L5" s="46"/>
+      <c r="M5" s="48"/>
+      <c r="N5" s="48"/>
     </row>
     <row r="6" spans="2:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="8" t="str">
@@ -3655,20 +3655,20 @@
       <c r="C6" s="8"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
-      <c r="F6" s="53" t="str">
+      <c r="F6" s="54" t="str">
         <f>IF(H5=Utileria!C30,"¿Cuál?","")</f>
         <v/>
       </c>
-      <c r="G6" s="53"/>
-      <c r="H6" s="44"/>
-      <c r="I6" s="44"/>
-      <c r="J6" s="44"/>
-      <c r="K6" s="45" t="s">
+      <c r="G6" s="54"/>
+      <c r="H6" s="45"/>
+      <c r="I6" s="45"/>
+      <c r="J6" s="45"/>
+      <c r="K6" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="L6" s="45"/>
-      <c r="M6" s="51"/>
-      <c r="N6" s="52"/>
+      <c r="L6" s="46"/>
+      <c r="M6" s="52"/>
+      <c r="N6" s="53"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B7" s="5"/>
@@ -3678,113 +3678,113 @@
       <c r="H7" s="5"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B8" s="48" t="s">
+      <c r="B8" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="48"/>
-      <c r="D8" s="49">
+      <c r="C8" s="49"/>
+      <c r="D8" s="50">
         <v>10</v>
       </c>
-      <c r="E8" s="49"/>
-      <c r="F8" s="49"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="50"/>
       <c r="H8" s="5"/>
-      <c r="I8" s="45" t="s">
+      <c r="I8" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="J8" s="45"/>
+      <c r="J8" s="46"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B9" s="53" t="str">
+      <c r="B9" s="54" t="str">
         <f>IF(D8=Utileria!E12,"¿Cuál?","")</f>
         <v/>
       </c>
-      <c r="C9" s="53"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="44"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="45"/>
       <c r="G9" s="35"/>
       <c r="H9" s="5"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="K10" s="50"/>
-      <c r="L10" s="50"/>
-      <c r="M10" s="50"/>
-      <c r="N10" s="50"/>
+      <c r="K10" s="51"/>
+      <c r="L10" s="51"/>
+      <c r="M10" s="51"/>
+      <c r="N10" s="51"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
-      <c r="F11" s="44"/>
-      <c r="G11" s="44"/>
-      <c r="H11" s="44"/>
-      <c r="K11" s="50"/>
-      <c r="L11" s="50"/>
-      <c r="M11" s="50"/>
-      <c r="N11" s="50"/>
+      <c r="F11" s="45"/>
+      <c r="G11" s="45"/>
+      <c r="H11" s="45"/>
+      <c r="K11" s="51"/>
+      <c r="L11" s="51"/>
+      <c r="M11" s="51"/>
+      <c r="N11" s="51"/>
     </row>
     <row r="12" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="46" t="s">
+      <c r="B12" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="46"/>
-      <c r="D12" s="54"/>
-      <c r="E12" s="54"/>
-      <c r="F12" s="54"/>
-      <c r="G12" s="54"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
       <c r="H12" s="7" t="s">
         <v>39</v>
       </c>
       <c r="I12" s="7"/>
-      <c r="J12" s="54"/>
-      <c r="K12" s="54"/>
-      <c r="L12" s="54"/>
-      <c r="M12" s="54"/>
-      <c r="N12" s="54"/>
+      <c r="J12" s="55"/>
+      <c r="K12" s="55"/>
+      <c r="L12" s="55"/>
+      <c r="M12" s="55"/>
+      <c r="N12" s="55"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B15" s="45" t="s">
+      <c r="B15" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="45"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="45"/>
-      <c r="F15" s="45"/>
-      <c r="G15" s="45"/>
-      <c r="H15" s="45"/>
-      <c r="I15" s="45"/>
-      <c r="J15" s="45"/>
-      <c r="K15" s="45"/>
-      <c r="L15" s="45"/>
-      <c r="M15" s="45"/>
-      <c r="N15" s="45"/>
+      <c r="C15" s="46"/>
+      <c r="D15" s="46"/>
+      <c r="E15" s="46"/>
+      <c r="F15" s="46"/>
+      <c r="G15" s="46"/>
+      <c r="H15" s="46"/>
+      <c r="I15" s="46"/>
+      <c r="J15" s="46"/>
+      <c r="K15" s="46"/>
+      <c r="L15" s="46"/>
+      <c r="M15" s="46"/>
+      <c r="N15" s="46"/>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B17" s="7" t="s">
         <v>10</v>
       </c>
       <c r="C17" s="7"/>
-      <c r="D17" s="50">
+      <c r="D17" s="51">
         <v>7</v>
       </c>
-      <c r="E17" s="50"/>
-      <c r="F17" s="50"/>
+      <c r="E17" s="51"/>
+      <c r="F17" s="51"/>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
       <c r="K17" s="7" t="s">
         <v>47</v>
       </c>
       <c r="L17" s="7"/>
-      <c r="M17" s="55"/>
-      <c r="N17" s="55"/>
+      <c r="M17" s="56"/>
+      <c r="N17" s="56"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B18" s="43" t="str">
+      <c r="B18" s="44" t="str">
         <f>IF(D17=Utileria!G9,"¿Cuál?","")</f>
         <v/>
       </c>
-      <c r="C18" s="43"/>
+      <c r="C18" s="44"/>
       <c r="D18" s="41"/>
       <c r="E18" s="42"/>
       <c r="F18" s="42"/>
@@ -3792,102 +3792,102 @@
       <c r="H18" s="42"/>
     </row>
     <row r="19" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="59" t="s">
+      <c r="B19" s="60" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="59"/>
-      <c r="D19" s="45" t="s">
+      <c r="C19" s="60"/>
+      <c r="D19" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="45"/>
-      <c r="F19" s="45"/>
-      <c r="G19" s="45"/>
-      <c r="H19" s="45"/>
-      <c r="I19" s="45"/>
-      <c r="J19" s="45"/>
-      <c r="K19" s="45"/>
-      <c r="L19" s="45"/>
-      <c r="M19" s="45"/>
-      <c r="N19" s="45"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="46"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="46"/>
+      <c r="I19" s="46"/>
+      <c r="J19" s="46"/>
+      <c r="K19" s="46"/>
+      <c r="L19" s="46"/>
+      <c r="M19" s="46"/>
+      <c r="N19" s="46"/>
     </row>
     <row r="20" spans="2:14" ht="317" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="59"/>
-      <c r="C20" s="59"/>
-      <c r="D20" s="62"/>
-      <c r="E20" s="62"/>
-      <c r="F20" s="62"/>
-      <c r="G20" s="62"/>
-      <c r="H20" s="62"/>
-      <c r="I20" s="62"/>
-      <c r="J20" s="62"/>
-      <c r="K20" s="62"/>
-      <c r="L20" s="62"/>
-      <c r="M20" s="62"/>
-      <c r="N20" s="62"/>
+      <c r="B20" s="60"/>
+      <c r="C20" s="60"/>
+      <c r="D20" s="63"/>
+      <c r="E20" s="63"/>
+      <c r="F20" s="63"/>
+      <c r="G20" s="63"/>
+      <c r="H20" s="63"/>
+      <c r="I20" s="63"/>
+      <c r="J20" s="63"/>
+      <c r="K20" s="63"/>
+      <c r="L20" s="63"/>
+      <c r="M20" s="63"/>
+      <c r="N20" s="63"/>
     </row>
     <row r="21" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="59"/>
-      <c r="C21" s="59"/>
-      <c r="D21" s="45" t="s">
+      <c r="B21" s="60"/>
+      <c r="C21" s="60"/>
+      <c r="D21" s="46" t="s">
         <v>65</v>
       </c>
-      <c r="E21" s="45"/>
-      <c r="F21" s="45"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="45"/>
-      <c r="I21" s="45"/>
-      <c r="J21" s="45"/>
-      <c r="K21" s="45"/>
-      <c r="L21" s="45"/>
-      <c r="M21" s="45"/>
-      <c r="N21" s="45"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="46"/>
+      <c r="I21" s="46"/>
+      <c r="J21" s="46"/>
+      <c r="K21" s="46"/>
+      <c r="L21" s="46"/>
+      <c r="M21" s="46"/>
+      <c r="N21" s="46"/>
     </row>
     <row r="22" spans="2:14" ht="409.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="59"/>
-      <c r="C22" s="59"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="60"/>
-      <c r="G22" s="60"/>
-      <c r="H22" s="60"/>
-      <c r="I22" s="60"/>
-      <c r="J22" s="60"/>
-      <c r="K22" s="60"/>
-      <c r="L22" s="60"/>
-      <c r="M22" s="60"/>
-      <c r="N22" s="60"/>
+      <c r="B22" s="60"/>
+      <c r="C22" s="60"/>
+      <c r="D22" s="61"/>
+      <c r="E22" s="61"/>
+      <c r="F22" s="61"/>
+      <c r="G22" s="61"/>
+      <c r="H22" s="61"/>
+      <c r="I22" s="61"/>
+      <c r="J22" s="61"/>
+      <c r="K22" s="61"/>
+      <c r="L22" s="61"/>
+      <c r="M22" s="61"/>
+      <c r="N22" s="61"/>
     </row>
     <row r="23" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="59"/>
-      <c r="C23" s="59"/>
-      <c r="D23" s="45" t="s">
+      <c r="B23" s="60"/>
+      <c r="C23" s="60"/>
+      <c r="D23" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="E23" s="45"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="45"/>
-      <c r="I23" s="45"/>
-      <c r="J23" s="45"/>
-      <c r="K23" s="45"/>
-      <c r="L23" s="45"/>
-      <c r="M23" s="45"/>
-      <c r="N23" s="45"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="46"/>
+      <c r="I23" s="46"/>
+      <c r="J23" s="46"/>
+      <c r="K23" s="46"/>
+      <c r="L23" s="46"/>
+      <c r="M23" s="46"/>
+      <c r="N23" s="46"/>
     </row>
     <row r="24" spans="2:14" ht="88.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="59"/>
-      <c r="C24" s="59"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
-      <c r="G24" s="60"/>
-      <c r="H24" s="60"/>
-      <c r="I24" s="60"/>
-      <c r="J24" s="60"/>
-      <c r="K24" s="60"/>
-      <c r="L24" s="60"/>
-      <c r="M24" s="60"/>
-      <c r="N24" s="60"/>
+      <c r="B24" s="60"/>
+      <c r="C24" s="60"/>
+      <c r="D24" s="61"/>
+      <c r="E24" s="61"/>
+      <c r="F24" s="61"/>
+      <c r="G24" s="61"/>
+      <c r="H24" s="61"/>
+      <c r="I24" s="61"/>
+      <c r="J24" s="61"/>
+      <c r="K24" s="61"/>
+      <c r="L24" s="61"/>
+      <c r="M24" s="61"/>
+      <c r="N24" s="61"/>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.35">
       <c r="D25" s="9"/>
@@ -3903,21 +3903,21 @@
       <c r="N25" s="9"/>
     </row>
     <row r="26" spans="2:14" ht="95.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="59" t="s">
+      <c r="B26" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="C26" s="59"/>
-      <c r="D26" s="58"/>
-      <c r="E26" s="58"/>
-      <c r="F26" s="58"/>
-      <c r="G26" s="58"/>
-      <c r="H26" s="58"/>
-      <c r="I26" s="58"/>
-      <c r="J26" s="58"/>
-      <c r="K26" s="58"/>
-      <c r="L26" s="58"/>
-      <c r="M26" s="58"/>
-      <c r="N26" s="58"/>
+      <c r="C26" s="60"/>
+      <c r="D26" s="59"/>
+      <c r="E26" s="59"/>
+      <c r="F26" s="59"/>
+      <c r="G26" s="59"/>
+      <c r="H26" s="59"/>
+      <c r="I26" s="59"/>
+      <c r="J26" s="59"/>
+      <c r="K26" s="59"/>
+      <c r="L26" s="59"/>
+      <c r="M26" s="59"/>
+      <c r="N26" s="59"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B27" s="5"/>
@@ -3935,154 +3935,154 @@
       <c r="N27" s="9"/>
     </row>
     <row r="28" spans="2:14" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="59" t="s">
+      <c r="B28" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="59"/>
-      <c r="D28" s="58"/>
-      <c r="E28" s="61"/>
-      <c r="F28" s="61"/>
-      <c r="G28" s="61"/>
-      <c r="H28" s="61"/>
-      <c r="I28" s="61"/>
-      <c r="J28" s="61"/>
-      <c r="K28" s="61"/>
-      <c r="L28" s="61"/>
-      <c r="M28" s="61"/>
-      <c r="N28" s="61"/>
+      <c r="C28" s="60"/>
+      <c r="D28" s="59"/>
+      <c r="E28" s="62"/>
+      <c r="F28" s="62"/>
+      <c r="G28" s="62"/>
+      <c r="H28" s="62"/>
+      <c r="I28" s="62"/>
+      <c r="J28" s="62"/>
+      <c r="K28" s="62"/>
+      <c r="L28" s="62"/>
+      <c r="M28" s="62"/>
+      <c r="N28" s="62"/>
     </row>
     <row r="29" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="30" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="45" t="s">
+      <c r="B30" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="C30" s="45"/>
-      <c r="D30" s="63"/>
-      <c r="E30" s="63"/>
-      <c r="F30" s="63"/>
-      <c r="G30" s="63"/>
-      <c r="H30" s="63"/>
-      <c r="I30" s="63"/>
-      <c r="J30" s="63"/>
-      <c r="K30" s="63"/>
-      <c r="L30" s="63"/>
-      <c r="M30" s="63"/>
-      <c r="N30" s="63"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="64"/>
+      <c r="E30" s="64"/>
+      <c r="F30" s="64"/>
+      <c r="G30" s="64"/>
+      <c r="H30" s="64"/>
+      <c r="I30" s="64"/>
+      <c r="J30" s="64"/>
+      <c r="K30" s="64"/>
+      <c r="L30" s="64"/>
+      <c r="M30" s="64"/>
+      <c r="N30" s="64"/>
     </row>
     <row r="31" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B31" s="11"/>
       <c r="C31" s="11"/>
-      <c r="D31" s="63"/>
-      <c r="E31" s="63"/>
-      <c r="F31" s="63"/>
-      <c r="G31" s="63"/>
-      <c r="H31" s="63"/>
-      <c r="I31" s="63"/>
-      <c r="J31" s="63"/>
-      <c r="K31" s="63"/>
-      <c r="L31" s="63"/>
-      <c r="M31" s="63"/>
-      <c r="N31" s="63"/>
+      <c r="D31" s="64"/>
+      <c r="E31" s="64"/>
+      <c r="F31" s="64"/>
+      <c r="G31" s="64"/>
+      <c r="H31" s="64"/>
+      <c r="I31" s="64"/>
+      <c r="J31" s="64"/>
+      <c r="K31" s="64"/>
+      <c r="L31" s="64"/>
+      <c r="M31" s="64"/>
+      <c r="N31" s="64"/>
     </row>
     <row r="32" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="12"/>
-      <c r="C32" s="57"/>
-      <c r="D32" s="57"/>
-      <c r="E32" s="57"/>
-      <c r="F32" s="57"/>
-      <c r="G32" s="57"/>
-      <c r="H32" s="57"/>
-      <c r="I32" s="57"/>
-      <c r="J32" s="57"/>
-      <c r="K32" s="57"/>
-      <c r="L32" s="57"/>
-      <c r="M32" s="57"/>
-      <c r="N32" s="57"/>
+      <c r="C32" s="58"/>
+      <c r="D32" s="58"/>
+      <c r="E32" s="58"/>
+      <c r="F32" s="58"/>
+      <c r="G32" s="58"/>
+      <c r="H32" s="58"/>
+      <c r="I32" s="58"/>
+      <c r="J32" s="58"/>
+      <c r="K32" s="58"/>
+      <c r="L32" s="58"/>
+      <c r="M32" s="58"/>
+      <c r="N32" s="58"/>
     </row>
     <row r="33" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="12"/>
-      <c r="C33" s="57"/>
-      <c r="D33" s="57"/>
-      <c r="E33" s="57"/>
-      <c r="F33" s="57"/>
-      <c r="G33" s="57"/>
-      <c r="H33" s="57"/>
-      <c r="I33" s="57"/>
-      <c r="J33" s="57"/>
-      <c r="K33" s="57"/>
-      <c r="L33" s="57"/>
-      <c r="M33" s="57"/>
-      <c r="N33" s="57"/>
+      <c r="C33" s="58"/>
+      <c r="D33" s="58"/>
+      <c r="E33" s="58"/>
+      <c r="F33" s="58"/>
+      <c r="G33" s="58"/>
+      <c r="H33" s="58"/>
+      <c r="I33" s="58"/>
+      <c r="J33" s="58"/>
+      <c r="K33" s="58"/>
+      <c r="L33" s="58"/>
+      <c r="M33" s="58"/>
+      <c r="N33" s="58"/>
     </row>
     <row r="34" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="35" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B35" s="45" t="s">
+      <c r="B35" s="46" t="s">
         <v>67</v>
       </c>
-      <c r="C35" s="45"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="45"/>
-      <c r="G35" s="45"/>
-      <c r="H35" s="45"/>
-      <c r="I35" s="45"/>
-      <c r="J35" s="45"/>
-      <c r="K35" s="45"/>
-      <c r="L35" s="45"/>
-      <c r="M35" s="45"/>
-      <c r="N35" s="45"/>
+      <c r="C35" s="46"/>
+      <c r="D35" s="46"/>
+      <c r="E35" s="46"/>
+      <c r="F35" s="46"/>
+      <c r="G35" s="46"/>
+      <c r="H35" s="46"/>
+      <c r="I35" s="46"/>
+      <c r="J35" s="46"/>
+      <c r="K35" s="46"/>
+      <c r="L35" s="46"/>
+      <c r="M35" s="46"/>
+      <c r="N35" s="46"/>
     </row>
     <row r="36" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="37" spans="2:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B37" s="46" t="s">
+      <c r="B37" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C37" s="46"/>
-      <c r="D37" s="54"/>
-      <c r="E37" s="54"/>
-      <c r="F37" s="54"/>
-      <c r="G37" s="54"/>
-      <c r="H37" s="45" t="s">
+      <c r="C37" s="47"/>
+      <c r="D37" s="55"/>
+      <c r="E37" s="55"/>
+      <c r="F37" s="55"/>
+      <c r="G37" s="55"/>
+      <c r="H37" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="I37" s="45"/>
-      <c r="J37" s="54"/>
-      <c r="K37" s="54"/>
-      <c r="L37" s="54"/>
-      <c r="M37" s="54"/>
+      <c r="I37" s="46"/>
+      <c r="J37" s="55"/>
+      <c r="K37" s="55"/>
+      <c r="L37" s="55"/>
+      <c r="M37" s="55"/>
     </row>
     <row r="38" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="39" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="45" t="s">
+      <c r="B39" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="C39" s="45"/>
-      <c r="D39" s="56"/>
-      <c r="E39" s="50"/>
-      <c r="F39" s="50"/>
-      <c r="G39" s="50"/>
-      <c r="H39" s="50"/>
-      <c r="I39" s="50"/>
-      <c r="J39" s="50"/>
-      <c r="K39" s="50"/>
-      <c r="L39" s="50"/>
-      <c r="M39" s="50"/>
-      <c r="N39" s="50"/>
+      <c r="C39" s="46"/>
+      <c r="D39" s="57"/>
+      <c r="E39" s="51"/>
+      <c r="F39" s="51"/>
+      <c r="G39" s="51"/>
+      <c r="H39" s="51"/>
+      <c r="I39" s="51"/>
+      <c r="J39" s="51"/>
+      <c r="K39" s="51"/>
+      <c r="L39" s="51"/>
+      <c r="M39" s="51"/>
+      <c r="N39" s="51"/>
     </row>
     <row r="40" spans="2:14" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B40" s="11"/>
       <c r="C40" s="11"/>
-      <c r="D40" s="50"/>
-      <c r="E40" s="50"/>
-      <c r="F40" s="50"/>
-      <c r="G40" s="50"/>
-      <c r="H40" s="50"/>
-      <c r="I40" s="50"/>
-      <c r="J40" s="50"/>
-      <c r="K40" s="50"/>
-      <c r="L40" s="50"/>
-      <c r="M40" s="50"/>
-      <c r="N40" s="50"/>
+      <c r="D40" s="51"/>
+      <c r="E40" s="51"/>
+      <c r="F40" s="51"/>
+      <c r="G40" s="51"/>
+      <c r="H40" s="51"/>
+      <c r="I40" s="51"/>
+      <c r="J40" s="51"/>
+      <c r="K40" s="51"/>
+      <c r="L40" s="51"/>
+      <c r="M40" s="51"/>
+      <c r="N40" s="51"/>
     </row>
     <row r="42" spans="2:14" ht="39" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
@@ -4311,122 +4311,122 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="65" t="s">
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="66" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="66" t="s">
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="66"/>
-      <c r="L2" s="67" t="s">
+      <c r="K2" s="67"/>
+      <c r="L2" s="68" t="s">
         <v>23</v>
       </c>
-      <c r="M2" s="67"/>
-      <c r="N2" s="67"/>
+      <c r="M2" s="68"/>
+      <c r="N2" s="68"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B3" s="64"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="65"/>
-      <c r="G3" s="65"/>
-      <c r="H3" s="65"/>
-      <c r="I3" s="65"/>
-      <c r="J3" s="66" t="s">
+      <c r="B3" s="65"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="66"/>
+      <c r="J3" s="67" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="66"/>
-      <c r="L3" s="67">
+      <c r="K3" s="67"/>
+      <c r="L3" s="68">
         <v>4</v>
       </c>
-      <c r="M3" s="67"/>
-      <c r="N3" s="67"/>
+      <c r="M3" s="68"/>
+      <c r="N3" s="68"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B4" s="64"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="64"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="65"/>
-      <c r="H4" s="65"/>
-      <c r="I4" s="65"/>
-      <c r="J4" s="66" t="s">
+      <c r="B4" s="65"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
+      <c r="H4" s="66"/>
+      <c r="I4" s="66"/>
+      <c r="J4" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="K4" s="66"/>
-      <c r="L4" s="67" t="s">
+      <c r="K4" s="67"/>
+      <c r="L4" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="M4" s="67"/>
-      <c r="N4" s="67"/>
+      <c r="M4" s="68"/>
+      <c r="N4" s="68"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B5" s="64"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="65"/>
-      <c r="F5" s="65"/>
-      <c r="G5" s="65"/>
-      <c r="H5" s="65"/>
-      <c r="I5" s="65"/>
-      <c r="J5" s="66" t="s">
+      <c r="B5" s="65"/>
+      <c r="C5" s="65"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
+      <c r="H5" s="66"/>
+      <c r="I5" s="66"/>
+      <c r="J5" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="K5" s="66"/>
-      <c r="L5" s="67" t="s">
+      <c r="K5" s="67"/>
+      <c r="L5" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="M5" s="67"/>
-      <c r="N5" s="67"/>
+      <c r="M5" s="68"/>
+      <c r="N5" s="68"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B7" s="45" t="s">
+      <c r="B7" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="45"/>
-      <c r="I7" s="45"/>
-      <c r="J7" s="45"/>
-      <c r="K7" s="45"/>
-      <c r="L7" s="45"/>
-      <c r="M7" s="45"/>
-      <c r="N7" s="45"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="46"/>
+      <c r="G7" s="46"/>
+      <c r="H7" s="46"/>
+      <c r="I7" s="46"/>
+      <c r="J7" s="46"/>
+      <c r="K7" s="46"/>
+      <c r="L7" s="46"/>
+      <c r="M7" s="46"/>
+      <c r="N7" s="46"/>
     </row>
     <row r="9" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C9" s="49"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
-      <c r="F9" s="46" t="s">
+      <c r="C9" s="50"/>
+      <c r="D9" s="50"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="G9" s="46"/>
-      <c r="H9" s="50">
+      <c r="G9" s="47"/>
+      <c r="H9" s="51">
         <v>1</v>
       </c>
-      <c r="I9" s="50"/>
-      <c r="J9" s="50"/>
-      <c r="K9" s="45" t="s">
+      <c r="I9" s="51"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="L9" s="45"/>
-      <c r="M9" s="47"/>
-      <c r="N9" s="47"/>
+      <c r="L9" s="46"/>
+      <c r="M9" s="48"/>
+      <c r="N9" s="48"/>
     </row>
     <row r="10" spans="2:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="5"/>
@@ -4435,15 +4435,15 @@
       <c r="E10" s="5"/>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
-      <c r="H10" s="69"/>
-      <c r="I10" s="69"/>
-      <c r="J10" s="69"/>
-      <c r="K10" s="45" t="s">
+      <c r="H10" s="70"/>
+      <c r="I10" s="70"/>
+      <c r="J10" s="70"/>
+      <c r="K10" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="L10" s="45"/>
-      <c r="M10" s="52"/>
-      <c r="N10" s="52"/>
+      <c r="L10" s="46"/>
+      <c r="M10" s="53"/>
+      <c r="N10" s="53"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B11" s="5"/>
@@ -4453,18 +4453,18 @@
       <c r="H11" s="5"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B12" s="48" t="s">
+      <c r="B12" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="48"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="49"/>
-      <c r="F12" s="49"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="50"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="50"/>
       <c r="H12" s="5"/>
-      <c r="I12" s="45" t="s">
+      <c r="I12" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="J12" s="45"/>
+      <c r="J12" s="46"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B13" s="5"/>
@@ -4476,10 +4476,10 @@
       <c r="H13" s="5"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="K14" s="50"/>
-      <c r="L14" s="50"/>
-      <c r="M14" s="50"/>
-      <c r="N14" s="50"/>
+      <c r="K14" s="51"/>
+      <c r="L14" s="51"/>
+      <c r="M14" s="51"/>
+      <c r="N14" s="51"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B15" s="5"/>
@@ -4489,206 +4489,206 @@
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
-      <c r="K15" s="50"/>
-      <c r="L15" s="50"/>
-      <c r="M15" s="50"/>
-      <c r="N15" s="50"/>
+      <c r="K15" s="51"/>
+      <c r="L15" s="51"/>
+      <c r="M15" s="51"/>
+      <c r="N15" s="51"/>
     </row>
     <row r="16" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="46" t="s">
+      <c r="B16" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="46"/>
-      <c r="D16" s="54"/>
-      <c r="E16" s="54"/>
-      <c r="F16" s="54"/>
-      <c r="G16" s="54"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="55"/>
+      <c r="E16" s="55"/>
+      <c r="F16" s="55"/>
+      <c r="G16" s="55"/>
       <c r="H16" s="7" t="s">
         <v>39</v>
       </c>
       <c r="I16" s="7"/>
-      <c r="J16" s="54"/>
-      <c r="K16" s="54"/>
-      <c r="L16" s="54"/>
-      <c r="M16" s="54"/>
-      <c r="N16" s="54"/>
+      <c r="J16" s="55"/>
+      <c r="K16" s="55"/>
+      <c r="L16" s="55"/>
+      <c r="M16" s="55"/>
+      <c r="N16" s="55"/>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B19" s="45" t="s">
+      <c r="B19" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="45"/>
-      <c r="D19" s="45"/>
-      <c r="E19" s="45"/>
-      <c r="F19" s="45"/>
-      <c r="G19" s="45"/>
-      <c r="H19" s="45"/>
-      <c r="I19" s="45"/>
-      <c r="J19" s="45"/>
-      <c r="K19" s="45"/>
-      <c r="L19" s="45"/>
-      <c r="M19" s="45"/>
-      <c r="N19" s="45"/>
+      <c r="C19" s="46"/>
+      <c r="D19" s="46"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="46"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="46"/>
+      <c r="I19" s="46"/>
+      <c r="J19" s="46"/>
+      <c r="K19" s="46"/>
+      <c r="L19" s="46"/>
+      <c r="M19" s="46"/>
+      <c r="N19" s="46"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B21" s="7" t="s">
         <v>10</v>
       </c>
       <c r="C21" s="7"/>
-      <c r="D21" s="50"/>
-      <c r="E21" s="50"/>
-      <c r="F21" s="50"/>
+      <c r="D21" s="51"/>
+      <c r="E21" s="51"/>
+      <c r="F21" s="51"/>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
       <c r="K21" s="7" t="s">
         <v>47</v>
       </c>
       <c r="L21" s="7"/>
-      <c r="M21" s="55"/>
-      <c r="N21" s="55"/>
+      <c r="M21" s="56"/>
+      <c r="N21" s="56"/>
     </row>
     <row r="23" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="59" t="s">
+      <c r="B23" s="60" t="s">
         <v>41</v>
       </c>
-      <c r="C23" s="59"/>
-      <c r="D23" s="45" t="s">
+      <c r="C23" s="60"/>
+      <c r="D23" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="45"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="45"/>
-      <c r="I23" s="45"/>
-      <c r="J23" s="45"/>
-      <c r="K23" s="45"/>
-      <c r="L23" s="45"/>
-      <c r="M23" s="45"/>
-      <c r="N23" s="45"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="46"/>
+      <c r="I23" s="46"/>
+      <c r="J23" s="46"/>
+      <c r="K23" s="46"/>
+      <c r="L23" s="46"/>
+      <c r="M23" s="46"/>
+      <c r="N23" s="46"/>
     </row>
     <row r="24" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="59"/>
-      <c r="C24" s="59"/>
-      <c r="D24" s="68"/>
-      <c r="E24" s="68"/>
-      <c r="F24" s="68"/>
-      <c r="G24" s="68"/>
-      <c r="H24" s="68"/>
-      <c r="I24" s="68"/>
-      <c r="J24" s="68"/>
-      <c r="K24" s="68"/>
-      <c r="L24" s="68"/>
-      <c r="M24" s="68"/>
-      <c r="N24" s="68"/>
+      <c r="B24" s="60"/>
+      <c r="C24" s="60"/>
+      <c r="D24" s="69"/>
+      <c r="E24" s="69"/>
+      <c r="F24" s="69"/>
+      <c r="G24" s="69"/>
+      <c r="H24" s="69"/>
+      <c r="I24" s="69"/>
+      <c r="J24" s="69"/>
+      <c r="K24" s="69"/>
+      <c r="L24" s="69"/>
+      <c r="M24" s="69"/>
+      <c r="N24" s="69"/>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B25" s="59"/>
-      <c r="C25" s="59"/>
-      <c r="D25" s="68"/>
-      <c r="E25" s="68"/>
-      <c r="F25" s="68"/>
-      <c r="G25" s="68"/>
-      <c r="H25" s="68"/>
-      <c r="I25" s="68"/>
-      <c r="J25" s="68"/>
-      <c r="K25" s="68"/>
-      <c r="L25" s="68"/>
-      <c r="M25" s="68"/>
-      <c r="N25" s="68"/>
+      <c r="B25" s="60"/>
+      <c r="C25" s="60"/>
+      <c r="D25" s="69"/>
+      <c r="E25" s="69"/>
+      <c r="F25" s="69"/>
+      <c r="G25" s="69"/>
+      <c r="H25" s="69"/>
+      <c r="I25" s="69"/>
+      <c r="J25" s="69"/>
+      <c r="K25" s="69"/>
+      <c r="L25" s="69"/>
+      <c r="M25" s="69"/>
+      <c r="N25" s="69"/>
     </row>
     <row r="26" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="59"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="45" t="s">
+      <c r="B26" s="60"/>
+      <c r="C26" s="60"/>
+      <c r="D26" s="46" t="s">
         <v>65</v>
       </c>
-      <c r="E26" s="45"/>
-      <c r="F26" s="45"/>
-      <c r="G26" s="45"/>
-      <c r="H26" s="45"/>
-      <c r="I26" s="45"/>
-      <c r="J26" s="45"/>
-      <c r="K26" s="45"/>
-      <c r="L26" s="45"/>
-      <c r="M26" s="45"/>
-      <c r="N26" s="45"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="46"/>
+      <c r="G26" s="46"/>
+      <c r="H26" s="46"/>
+      <c r="I26" s="46"/>
+      <c r="J26" s="46"/>
+      <c r="K26" s="46"/>
+      <c r="L26" s="46"/>
+      <c r="M26" s="46"/>
+      <c r="N26" s="46"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B27" s="59"/>
-      <c r="C27" s="59"/>
-      <c r="D27" s="68"/>
-      <c r="E27" s="68"/>
-      <c r="F27" s="68"/>
-      <c r="G27" s="68"/>
-      <c r="H27" s="68"/>
-      <c r="I27" s="68"/>
-      <c r="J27" s="68"/>
-      <c r="K27" s="68"/>
-      <c r="L27" s="68"/>
-      <c r="M27" s="68"/>
-      <c r="N27" s="68"/>
+      <c r="B27" s="60"/>
+      <c r="C27" s="60"/>
+      <c r="D27" s="69"/>
+      <c r="E27" s="69"/>
+      <c r="F27" s="69"/>
+      <c r="G27" s="69"/>
+      <c r="H27" s="69"/>
+      <c r="I27" s="69"/>
+      <c r="J27" s="69"/>
+      <c r="K27" s="69"/>
+      <c r="L27" s="69"/>
+      <c r="M27" s="69"/>
+      <c r="N27" s="69"/>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B28" s="59"/>
-      <c r="C28" s="59"/>
-      <c r="D28" s="68"/>
-      <c r="E28" s="68"/>
-      <c r="F28" s="68"/>
-      <c r="G28" s="68"/>
-      <c r="H28" s="68"/>
-      <c r="I28" s="68"/>
-      <c r="J28" s="68"/>
-      <c r="K28" s="68"/>
-      <c r="L28" s="68"/>
-      <c r="M28" s="68"/>
-      <c r="N28" s="68"/>
+      <c r="B28" s="60"/>
+      <c r="C28" s="60"/>
+      <c r="D28" s="69"/>
+      <c r="E28" s="69"/>
+      <c r="F28" s="69"/>
+      <c r="G28" s="69"/>
+      <c r="H28" s="69"/>
+      <c r="I28" s="69"/>
+      <c r="J28" s="69"/>
+      <c r="K28" s="69"/>
+      <c r="L28" s="69"/>
+      <c r="M28" s="69"/>
+      <c r="N28" s="69"/>
     </row>
     <row r="29" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="59"/>
-      <c r="C29" s="59"/>
-      <c r="D29" s="45" t="s">
+      <c r="B29" s="60"/>
+      <c r="C29" s="60"/>
+      <c r="D29" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="E29" s="45"/>
-      <c r="F29" s="45"/>
-      <c r="G29" s="45"/>
-      <c r="H29" s="45"/>
-      <c r="I29" s="45"/>
-      <c r="J29" s="45"/>
-      <c r="K29" s="45"/>
-      <c r="L29" s="45"/>
-      <c r="M29" s="45"/>
-      <c r="N29" s="45"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="46"/>
+      <c r="G29" s="46"/>
+      <c r="H29" s="46"/>
+      <c r="I29" s="46"/>
+      <c r="J29" s="46"/>
+      <c r="K29" s="46"/>
+      <c r="L29" s="46"/>
+      <c r="M29" s="46"/>
+      <c r="N29" s="46"/>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B30" s="59"/>
-      <c r="C30" s="59"/>
-      <c r="D30" s="68"/>
-      <c r="E30" s="68"/>
-      <c r="F30" s="68"/>
-      <c r="G30" s="68"/>
-      <c r="H30" s="68"/>
-      <c r="I30" s="68"/>
-      <c r="J30" s="68"/>
-      <c r="K30" s="68"/>
-      <c r="L30" s="68"/>
-      <c r="M30" s="68"/>
-      <c r="N30" s="68"/>
+      <c r="B30" s="60"/>
+      <c r="C30" s="60"/>
+      <c r="D30" s="69"/>
+      <c r="E30" s="69"/>
+      <c r="F30" s="69"/>
+      <c r="G30" s="69"/>
+      <c r="H30" s="69"/>
+      <c r="I30" s="69"/>
+      <c r="J30" s="69"/>
+      <c r="K30" s="69"/>
+      <c r="L30" s="69"/>
+      <c r="M30" s="69"/>
+      <c r="N30" s="69"/>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B31" s="59"/>
-      <c r="C31" s="59"/>
-      <c r="D31" s="68"/>
-      <c r="E31" s="68"/>
-      <c r="F31" s="68"/>
-      <c r="G31" s="68"/>
-      <c r="H31" s="68"/>
-      <c r="I31" s="68"/>
-      <c r="J31" s="68"/>
-      <c r="K31" s="68"/>
-      <c r="L31" s="68"/>
-      <c r="M31" s="68"/>
-      <c r="N31" s="68"/>
+      <c r="B31" s="60"/>
+      <c r="C31" s="60"/>
+      <c r="D31" s="69"/>
+      <c r="E31" s="69"/>
+      <c r="F31" s="69"/>
+      <c r="G31" s="69"/>
+      <c r="H31" s="69"/>
+      <c r="I31" s="69"/>
+      <c r="J31" s="69"/>
+      <c r="K31" s="69"/>
+      <c r="L31" s="69"/>
+      <c r="M31" s="69"/>
+      <c r="N31" s="69"/>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.35">
       <c r="D32" s="9"/>
@@ -4704,53 +4704,53 @@
       <c r="N32" s="9"/>
     </row>
     <row r="33" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="59" t="s">
+      <c r="B33" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="C33" s="59"/>
-      <c r="D33" s="58" t="s">
+      <c r="C33" s="60"/>
+      <c r="D33" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="E33" s="58"/>
-      <c r="F33" s="58"/>
-      <c r="G33" s="58"/>
-      <c r="H33" s="58"/>
-      <c r="I33" s="58"/>
-      <c r="J33" s="58"/>
-      <c r="K33" s="58"/>
-      <c r="L33" s="58"/>
-      <c r="M33" s="58"/>
-      <c r="N33" s="58"/>
+      <c r="E33" s="59"/>
+      <c r="F33" s="59"/>
+      <c r="G33" s="59"/>
+      <c r="H33" s="59"/>
+      <c r="I33" s="59"/>
+      <c r="J33" s="59"/>
+      <c r="K33" s="59"/>
+      <c r="L33" s="59"/>
+      <c r="M33" s="59"/>
+      <c r="N33" s="59"/>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B34" s="59"/>
-      <c r="C34" s="59"/>
-      <c r="D34" s="58"/>
-      <c r="E34" s="58"/>
-      <c r="F34" s="58"/>
-      <c r="G34" s="58"/>
-      <c r="H34" s="58"/>
-      <c r="I34" s="58"/>
-      <c r="J34" s="58"/>
-      <c r="K34" s="58"/>
-      <c r="L34" s="58"/>
-      <c r="M34" s="58"/>
-      <c r="N34" s="58"/>
+      <c r="B34" s="60"/>
+      <c r="C34" s="60"/>
+      <c r="D34" s="59"/>
+      <c r="E34" s="59"/>
+      <c r="F34" s="59"/>
+      <c r="G34" s="59"/>
+      <c r="H34" s="59"/>
+      <c r="I34" s="59"/>
+      <c r="J34" s="59"/>
+      <c r="K34" s="59"/>
+      <c r="L34" s="59"/>
+      <c r="M34" s="59"/>
+      <c r="N34" s="59"/>
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B35" s="59"/>
-      <c r="C35" s="59"/>
-      <c r="D35" s="58"/>
-      <c r="E35" s="58"/>
-      <c r="F35" s="58"/>
-      <c r="G35" s="58"/>
-      <c r="H35" s="58"/>
-      <c r="I35" s="58"/>
-      <c r="J35" s="58"/>
-      <c r="K35" s="58"/>
-      <c r="L35" s="58"/>
-      <c r="M35" s="58"/>
-      <c r="N35" s="58"/>
+      <c r="B35" s="60"/>
+      <c r="C35" s="60"/>
+      <c r="D35" s="59"/>
+      <c r="E35" s="59"/>
+      <c r="F35" s="59"/>
+      <c r="G35" s="59"/>
+      <c r="H35" s="59"/>
+      <c r="I35" s="59"/>
+      <c r="J35" s="59"/>
+      <c r="K35" s="59"/>
+      <c r="L35" s="59"/>
+      <c r="M35" s="59"/>
+      <c r="N35" s="59"/>
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B36" s="5"/>
@@ -4768,186 +4768,186 @@
       <c r="N36" s="9"/>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B37" s="59" t="s">
+      <c r="B37" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C37" s="59"/>
-      <c r="D37" s="58" t="s">
+      <c r="C37" s="60"/>
+      <c r="D37" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="E37" s="61"/>
-      <c r="F37" s="61"/>
-      <c r="G37" s="61"/>
-      <c r="H37" s="61"/>
-      <c r="I37" s="61"/>
-      <c r="J37" s="61"/>
-      <c r="K37" s="61"/>
-      <c r="L37" s="61"/>
-      <c r="M37" s="61"/>
-      <c r="N37" s="61"/>
+      <c r="E37" s="62"/>
+      <c r="F37" s="62"/>
+      <c r="G37" s="62"/>
+      <c r="H37" s="62"/>
+      <c r="I37" s="62"/>
+      <c r="J37" s="62"/>
+      <c r="K37" s="62"/>
+      <c r="L37" s="62"/>
+      <c r="M37" s="62"/>
+      <c r="N37" s="62"/>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B38" s="59"/>
-      <c r="C38" s="59"/>
-      <c r="D38" s="61"/>
-      <c r="E38" s="61"/>
-      <c r="F38" s="61"/>
-      <c r="G38" s="61"/>
-      <c r="H38" s="61"/>
-      <c r="I38" s="61"/>
-      <c r="J38" s="61"/>
-      <c r="K38" s="61"/>
-      <c r="L38" s="61"/>
-      <c r="M38" s="61"/>
-      <c r="N38" s="61"/>
+      <c r="B38" s="60"/>
+      <c r="C38" s="60"/>
+      <c r="D38" s="62"/>
+      <c r="E38" s="62"/>
+      <c r="F38" s="62"/>
+      <c r="G38" s="62"/>
+      <c r="H38" s="62"/>
+      <c r="I38" s="62"/>
+      <c r="J38" s="62"/>
+      <c r="K38" s="62"/>
+      <c r="L38" s="62"/>
+      <c r="M38" s="62"/>
+      <c r="N38" s="62"/>
     </row>
     <row r="39" spans="2:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="40" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="45" t="s">
+      <c r="B40" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="C40" s="45"/>
-      <c r="D40" s="70" t="str">
+      <c r="C40" s="46"/>
+      <c r="D40" s="71" t="str">
         <f>IF($H$9=1,Utileria!$L$15,IF($H$9=2,Utileria!$L$15,IF($H$9=3,Utileria!$L$15,IF($H$9=7,Utileria!L$15,IF($H$9=8,Utileria!$L$15,IF($H$9=16,Utileria!$L$15,IF($H$9=17,Utileria!$L$15,IF($H$9=19,Utileria!$L$15,IF($H$9=24,Utileria!$L$15,IF($H$9=25,Utileria!$L$15,""))))))))))</f>
         <v>¡ATENCIÓN! Para que tu solicitud sea atendida es necesario adjuntar los insumos que a continuación se muestran, en caso de no hacerlo, se puede incurrir en retrasos.</v>
       </c>
-      <c r="E40" s="70"/>
-      <c r="F40" s="70"/>
-      <c r="G40" s="70"/>
-      <c r="H40" s="70"/>
-      <c r="I40" s="70"/>
-      <c r="J40" s="70"/>
-      <c r="K40" s="70"/>
-      <c r="L40" s="70"/>
-      <c r="M40" s="70"/>
-      <c r="N40" s="70"/>
+      <c r="E40" s="71"/>
+      <c r="F40" s="71"/>
+      <c r="G40" s="71"/>
+      <c r="H40" s="71"/>
+      <c r="I40" s="71"/>
+      <c r="J40" s="71"/>
+      <c r="K40" s="71"/>
+      <c r="L40" s="71"/>
+      <c r="M40" s="71"/>
+      <c r="N40" s="71"/>
     </row>
     <row r="41" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B41" s="11"/>
       <c r="C41" s="11"/>
-      <c r="D41" s="70"/>
-      <c r="E41" s="70"/>
-      <c r="F41" s="70"/>
-      <c r="G41" s="70"/>
-      <c r="H41" s="70"/>
-      <c r="I41" s="70"/>
-      <c r="J41" s="70"/>
-      <c r="K41" s="70"/>
-      <c r="L41" s="70"/>
-      <c r="M41" s="70"/>
-      <c r="N41" s="70"/>
+      <c r="D41" s="71"/>
+      <c r="E41" s="71"/>
+      <c r="F41" s="71"/>
+      <c r="G41" s="71"/>
+      <c r="H41" s="71"/>
+      <c r="I41" s="71"/>
+      <c r="J41" s="71"/>
+      <c r="K41" s="71"/>
+      <c r="L41" s="71"/>
+      <c r="M41" s="71"/>
+      <c r="N41" s="71"/>
     </row>
     <row r="42" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B42" s="12">
         <f>IF(C42="","", 1)</f>
         <v>1</v>
       </c>
-      <c r="C42" s="57" t="str">
+      <c r="C42" s="58" t="str">
         <f>IF($H$9=1,Utileria!$L$9,IF($H$9=2,Utileria!$L$12,IF($H$9=3,Utileria!$L$11,IF($H$9=7,Utileria!L$6,IF($H$9=8,Utileria!$L$6,IF($H$9=16,Utileria!$L$5,IF($H$9=17,Utileria!$L$4,IF($H$9=19,Utileria!$L$4,IF($H$9=24,Utileria!$L$4,IF($H$9=25,Utileria!$L$4,"N/A"))))))))))</f>
         <v>Usuario y contraseña</v>
       </c>
-      <c r="D42" s="57"/>
-      <c r="E42" s="57"/>
-      <c r="F42" s="57"/>
-      <c r="G42" s="57"/>
-      <c r="H42" s="57"/>
-      <c r="I42" s="57"/>
-      <c r="J42" s="57"/>
-      <c r="K42" s="57"/>
-      <c r="L42" s="57"/>
-      <c r="M42" s="57"/>
-      <c r="N42" s="57"/>
+      <c r="D42" s="58"/>
+      <c r="E42" s="58"/>
+      <c r="F42" s="58"/>
+      <c r="G42" s="58"/>
+      <c r="H42" s="58"/>
+      <c r="I42" s="58"/>
+      <c r="J42" s="58"/>
+      <c r="K42" s="58"/>
+      <c r="L42" s="58"/>
+      <c r="M42" s="58"/>
+      <c r="N42" s="58"/>
     </row>
     <row r="43" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B43" s="12">
         <f>IF(C43="","", 2)</f>
         <v>2</v>
       </c>
-      <c r="C43" s="57" t="str">
+      <c r="C43" s="58" t="str">
         <f>IF($H$9=1,Utileria!$L$10,IF($H$9=7,Utileria!$L$8,IF($H$9=8,Utileria!$L$7,IF($H$9=2,Utileria!$L$13,""))))</f>
         <v>Folio ligado al usuario, adicional ese folio debe de contener datos del miembro de QA.</v>
       </c>
-      <c r="D43" s="57"/>
-      <c r="E43" s="57"/>
-      <c r="F43" s="57"/>
-      <c r="G43" s="57"/>
-      <c r="H43" s="57"/>
-      <c r="I43" s="57"/>
-      <c r="J43" s="57"/>
-      <c r="K43" s="57"/>
-      <c r="L43" s="57"/>
-      <c r="M43" s="57"/>
-      <c r="N43" s="57"/>
+      <c r="D43" s="58"/>
+      <c r="E43" s="58"/>
+      <c r="F43" s="58"/>
+      <c r="G43" s="58"/>
+      <c r="H43" s="58"/>
+      <c r="I43" s="58"/>
+      <c r="J43" s="58"/>
+      <c r="K43" s="58"/>
+      <c r="L43" s="58"/>
+      <c r="M43" s="58"/>
+      <c r="N43" s="58"/>
     </row>
     <row r="44" spans="2:14" ht="26.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="45" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B45" s="45" t="s">
+      <c r="B45" s="46" t="s">
         <v>67</v>
       </c>
-      <c r="C45" s="45"/>
-      <c r="D45" s="45"/>
-      <c r="E45" s="45"/>
-      <c r="F45" s="45"/>
-      <c r="G45" s="45"/>
-      <c r="H45" s="45"/>
-      <c r="I45" s="45"/>
-      <c r="J45" s="45"/>
-      <c r="K45" s="45"/>
-      <c r="L45" s="45"/>
-      <c r="M45" s="45"/>
-      <c r="N45" s="45"/>
+      <c r="C45" s="46"/>
+      <c r="D45" s="46"/>
+      <c r="E45" s="46"/>
+      <c r="F45" s="46"/>
+      <c r="G45" s="46"/>
+      <c r="H45" s="46"/>
+      <c r="I45" s="46"/>
+      <c r="J45" s="46"/>
+      <c r="K45" s="46"/>
+      <c r="L45" s="46"/>
+      <c r="M45" s="46"/>
+      <c r="N45" s="46"/>
     </row>
     <row r="46" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="47" spans="2:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B47" s="46" t="s">
+      <c r="B47" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C47" s="46"/>
-      <c r="D47" s="54"/>
-      <c r="E47" s="54"/>
-      <c r="F47" s="54"/>
-      <c r="G47" s="54"/>
-      <c r="H47" s="45" t="s">
+      <c r="C47" s="47"/>
+      <c r="D47" s="55"/>
+      <c r="E47" s="55"/>
+      <c r="F47" s="55"/>
+      <c r="G47" s="55"/>
+      <c r="H47" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="I47" s="45"/>
-      <c r="J47" s="54"/>
-      <c r="K47" s="54"/>
-      <c r="L47" s="54"/>
-      <c r="M47" s="54"/>
+      <c r="I47" s="46"/>
+      <c r="J47" s="55"/>
+      <c r="K47" s="55"/>
+      <c r="L47" s="55"/>
+      <c r="M47" s="55"/>
     </row>
     <row r="48" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="49" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B49" s="48" t="s">
+      <c r="B49" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="C49" s="48"/>
-      <c r="D49" s="50"/>
-      <c r="E49" s="50"/>
-      <c r="F49" s="50"/>
-      <c r="G49" s="50"/>
-      <c r="H49" s="50"/>
-      <c r="I49" s="50"/>
-      <c r="J49" s="50"/>
-      <c r="K49" s="50"/>
-      <c r="L49" s="50"/>
-      <c r="M49" s="50"/>
-      <c r="N49" s="50"/>
+      <c r="C49" s="49"/>
+      <c r="D49" s="51"/>
+      <c r="E49" s="51"/>
+      <c r="F49" s="51"/>
+      <c r="G49" s="51"/>
+      <c r="H49" s="51"/>
+      <c r="I49" s="51"/>
+      <c r="J49" s="51"/>
+      <c r="K49" s="51"/>
+      <c r="L49" s="51"/>
+      <c r="M49" s="51"/>
+      <c r="N49" s="51"/>
     </row>
     <row r="50" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B50" s="48"/>
-      <c r="C50" s="48"/>
-      <c r="D50" s="50"/>
-      <c r="E50" s="50"/>
-      <c r="F50" s="50"/>
-      <c r="G50" s="50"/>
-      <c r="H50" s="50"/>
-      <c r="I50" s="50"/>
-      <c r="J50" s="50"/>
-      <c r="K50" s="50"/>
-      <c r="L50" s="50"/>
-      <c r="M50" s="50"/>
-      <c r="N50" s="50"/>
+      <c r="B50" s="49"/>
+      <c r="C50" s="49"/>
+      <c r="D50" s="51"/>
+      <c r="E50" s="51"/>
+      <c r="F50" s="51"/>
+      <c r="G50" s="51"/>
+      <c r="H50" s="51"/>
+      <c r="I50" s="51"/>
+      <c r="J50" s="51"/>
+      <c r="K50" s="51"/>
+      <c r="L50" s="51"/>
+      <c r="M50" s="51"/>
+      <c r="N50" s="51"/>
     </row>
     <row r="51" spans="2:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B51" s="11"/>
@@ -5185,122 +5185,122 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="65" t="s">
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="66" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="66" t="s">
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="66"/>
-      <c r="L2" s="67" t="s">
+      <c r="K2" s="67"/>
+      <c r="L2" s="68" t="s">
         <v>23</v>
       </c>
-      <c r="M2" s="67"/>
-      <c r="N2" s="67"/>
+      <c r="M2" s="68"/>
+      <c r="N2" s="68"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B3" s="64"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="65"/>
-      <c r="G3" s="65"/>
-      <c r="H3" s="65"/>
-      <c r="I3" s="65"/>
-      <c r="J3" s="66" t="s">
+      <c r="B3" s="65"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="66"/>
+      <c r="J3" s="67" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="66"/>
-      <c r="L3" s="67">
+      <c r="K3" s="67"/>
+      <c r="L3" s="68">
         <v>4</v>
       </c>
-      <c r="M3" s="67"/>
-      <c r="N3" s="67"/>
+      <c r="M3" s="68"/>
+      <c r="N3" s="68"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B4" s="64"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="64"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="65"/>
-      <c r="H4" s="65"/>
-      <c r="I4" s="65"/>
-      <c r="J4" s="66" t="s">
+      <c r="B4" s="65"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
+      <c r="H4" s="66"/>
+      <c r="I4" s="66"/>
+      <c r="J4" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="K4" s="66"/>
-      <c r="L4" s="67" t="s">
+      <c r="K4" s="67"/>
+      <c r="L4" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="M4" s="67"/>
-      <c r="N4" s="67"/>
+      <c r="M4" s="68"/>
+      <c r="N4" s="68"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B5" s="64"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="65"/>
-      <c r="F5" s="65"/>
-      <c r="G5" s="65"/>
-      <c r="H5" s="65"/>
-      <c r="I5" s="65"/>
-      <c r="J5" s="66" t="s">
+      <c r="B5" s="65"/>
+      <c r="C5" s="65"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
+      <c r="H5" s="66"/>
+      <c r="I5" s="66"/>
+      <c r="J5" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="K5" s="66"/>
-      <c r="L5" s="67" t="s">
+      <c r="K5" s="67"/>
+      <c r="L5" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="M5" s="67"/>
-      <c r="N5" s="67"/>
+      <c r="M5" s="68"/>
+      <c r="N5" s="68"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B7" s="45" t="s">
+      <c r="B7" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="45"/>
-      <c r="I7" s="45"/>
-      <c r="J7" s="45"/>
-      <c r="K7" s="45"/>
-      <c r="L7" s="45"/>
-      <c r="M7" s="45"/>
-      <c r="N7" s="45"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="46"/>
+      <c r="G7" s="46"/>
+      <c r="H7" s="46"/>
+      <c r="I7" s="46"/>
+      <c r="J7" s="46"/>
+      <c r="K7" s="46"/>
+      <c r="L7" s="46"/>
+      <c r="M7" s="46"/>
+      <c r="N7" s="46"/>
     </row>
     <row r="9" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C9" s="49"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
-      <c r="F9" s="46" t="s">
+      <c r="C9" s="50"/>
+      <c r="D9" s="50"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="G9" s="46"/>
+      <c r="G9" s="47"/>
       <c r="H9" s="5">
         <v>17</v>
       </c>
-      <c r="K9" s="45" t="s">
+      <c r="K9" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="L9" s="45"/>
-      <c r="M9" s="72">
+      <c r="L9" s="46"/>
+      <c r="M9" s="73">
         <v>44577</v>
       </c>
-      <c r="N9" s="72"/>
+      <c r="N9" s="73"/>
     </row>
     <row r="10" spans="2:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="5"/>
@@ -5309,17 +5309,17 @@
       <c r="E10" s="5"/>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
-      <c r="H10" s="69"/>
-      <c r="I10" s="69"/>
-      <c r="J10" s="69"/>
-      <c r="K10" s="45" t="s">
+      <c r="H10" s="70"/>
+      <c r="I10" s="70"/>
+      <c r="J10" s="70"/>
+      <c r="K10" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="L10" s="45"/>
-      <c r="M10" s="73" t="s">
+      <c r="L10" s="46"/>
+      <c r="M10" s="74" t="s">
         <v>34</v>
       </c>
-      <c r="N10" s="73"/>
+      <c r="N10" s="74"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B11" s="5"/>
@@ -5331,18 +5331,18 @@
       </c>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B12" s="71" t="s">
+      <c r="B12" s="72" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="71"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="49"/>
-      <c r="F12" s="49"/>
+      <c r="C12" s="72"/>
+      <c r="D12" s="50"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="50"/>
       <c r="H12" s="5"/>
-      <c r="I12" s="45" t="s">
+      <c r="I12" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="J12" s="45"/>
+      <c r="J12" s="46"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B13" s="5"/>
@@ -5354,10 +5354,10 @@
       <c r="H13" s="5"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="K14" s="50"/>
-      <c r="L14" s="50"/>
-      <c r="M14" s="50"/>
-      <c r="N14" s="50"/>
+      <c r="K14" s="51"/>
+      <c r="L14" s="51"/>
+      <c r="M14" s="51"/>
+      <c r="N14" s="51"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B15" s="5"/>
@@ -5367,173 +5367,173 @@
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
-      <c r="K15" s="50"/>
-      <c r="L15" s="50"/>
-      <c r="M15" s="50"/>
-      <c r="N15" s="50"/>
+      <c r="K15" s="51"/>
+      <c r="L15" s="51"/>
+      <c r="M15" s="51"/>
+      <c r="N15" s="51"/>
     </row>
     <row r="16" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="46" t="s">
+      <c r="B16" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="46"/>
-      <c r="D16" s="74" t="s">
+      <c r="C16" s="47"/>
+      <c r="D16" s="75" t="s">
         <v>69</v>
       </c>
-      <c r="E16" s="74"/>
-      <c r="F16" s="74"/>
-      <c r="G16" s="74"/>
+      <c r="E16" s="75"/>
+      <c r="F16" s="75"/>
+      <c r="G16" s="75"/>
       <c r="H16" s="7" t="s">
         <v>39</v>
       </c>
       <c r="I16" s="7"/>
-      <c r="J16" s="74" t="s">
+      <c r="J16" s="75" t="s">
         <v>89</v>
       </c>
-      <c r="K16" s="74"/>
-      <c r="L16" s="74"/>
-      <c r="M16" s="74"/>
-      <c r="N16" s="74"/>
+      <c r="K16" s="75"/>
+      <c r="L16" s="75"/>
+      <c r="M16" s="75"/>
+      <c r="N16" s="75"/>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B19" s="45" t="s">
+      <c r="B19" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="45"/>
-      <c r="D19" s="45"/>
-      <c r="E19" s="45"/>
-      <c r="F19" s="45"/>
-      <c r="G19" s="45"/>
-      <c r="H19" s="45"/>
-      <c r="I19" s="45"/>
-      <c r="J19" s="45"/>
-      <c r="K19" s="45"/>
-      <c r="L19" s="45"/>
-      <c r="M19" s="45"/>
-      <c r="N19" s="45"/>
+      <c r="C19" s="46"/>
+      <c r="D19" s="46"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="46"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="46"/>
+      <c r="I19" s="46"/>
+      <c r="J19" s="46"/>
+      <c r="K19" s="46"/>
+      <c r="L19" s="46"/>
+      <c r="M19" s="46"/>
+      <c r="N19" s="46"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B21" s="7" t="s">
         <v>10</v>
       </c>
       <c r="C21" s="7"/>
-      <c r="D21" s="50"/>
-      <c r="E21" s="50"/>
-      <c r="F21" s="50"/>
+      <c r="D21" s="51"/>
+      <c r="E21" s="51"/>
+      <c r="F21" s="51"/>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
       <c r="K21" s="7" t="s">
         <v>47</v>
       </c>
       <c r="L21" s="7"/>
-      <c r="M21" s="73" t="s">
+      <c r="M21" s="74" t="s">
         <v>35</v>
       </c>
-      <c r="N21" s="73"/>
+      <c r="N21" s="74"/>
     </row>
     <row r="23" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="59" t="s">
+      <c r="B23" s="60" t="s">
         <v>41</v>
       </c>
-      <c r="C23" s="59"/>
-      <c r="D23" s="45" t="s">
+      <c r="C23" s="60"/>
+      <c r="D23" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="45"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="45"/>
-      <c r="I23" s="45"/>
-      <c r="J23" s="45"/>
-      <c r="K23" s="45"/>
-      <c r="L23" s="45"/>
-      <c r="M23" s="45"/>
-      <c r="N23" s="45"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="46"/>
+      <c r="I23" s="46"/>
+      <c r="J23" s="46"/>
+      <c r="K23" s="46"/>
+      <c r="L23" s="46"/>
+      <c r="M23" s="46"/>
+      <c r="N23" s="46"/>
     </row>
     <row r="24" spans="2:14" ht="123" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="59"/>
-      <c r="C24" s="59"/>
-      <c r="D24" s="75" t="s">
+      <c r="B24" s="60"/>
+      <c r="C24" s="60"/>
+      <c r="D24" s="76" t="s">
         <v>70</v>
       </c>
-      <c r="E24" s="75"/>
-      <c r="F24" s="75"/>
-      <c r="G24" s="75"/>
-      <c r="H24" s="75"/>
-      <c r="I24" s="75"/>
-      <c r="J24" s="75"/>
-      <c r="K24" s="75"/>
-      <c r="L24" s="75"/>
-      <c r="M24" s="75"/>
-      <c r="N24" s="75"/>
+      <c r="E24" s="76"/>
+      <c r="F24" s="76"/>
+      <c r="G24" s="76"/>
+      <c r="H24" s="76"/>
+      <c r="I24" s="76"/>
+      <c r="J24" s="76"/>
+      <c r="K24" s="76"/>
+      <c r="L24" s="76"/>
+      <c r="M24" s="76"/>
+      <c r="N24" s="76"/>
     </row>
     <row r="25" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="59"/>
-      <c r="C25" s="59"/>
-      <c r="D25" s="45" t="s">
+      <c r="B25" s="60"/>
+      <c r="C25" s="60"/>
+      <c r="D25" s="46" t="s">
         <v>65</v>
       </c>
-      <c r="E25" s="45"/>
-      <c r="F25" s="45"/>
-      <c r="G25" s="45"/>
-      <c r="H25" s="45"/>
-      <c r="I25" s="45"/>
-      <c r="J25" s="45"/>
-      <c r="K25" s="45"/>
-      <c r="L25" s="45"/>
-      <c r="M25" s="45"/>
-      <c r="N25" s="45"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="46"/>
+      <c r="G25" s="46"/>
+      <c r="H25" s="46"/>
+      <c r="I25" s="46"/>
+      <c r="J25" s="46"/>
+      <c r="K25" s="46"/>
+      <c r="L25" s="46"/>
+      <c r="M25" s="46"/>
+      <c r="N25" s="46"/>
     </row>
     <row r="26" spans="2:14" ht="363.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="59"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="75" t="s">
+      <c r="B26" s="60"/>
+      <c r="C26" s="60"/>
+      <c r="D26" s="76" t="s">
         <v>71</v>
       </c>
-      <c r="E26" s="75"/>
-      <c r="F26" s="75"/>
-      <c r="G26" s="75"/>
-      <c r="H26" s="75"/>
-      <c r="I26" s="75"/>
-      <c r="J26" s="75"/>
-      <c r="K26" s="75"/>
-      <c r="L26" s="75"/>
-      <c r="M26" s="75"/>
-      <c r="N26" s="75"/>
+      <c r="E26" s="76"/>
+      <c r="F26" s="76"/>
+      <c r="G26" s="76"/>
+      <c r="H26" s="76"/>
+      <c r="I26" s="76"/>
+      <c r="J26" s="76"/>
+      <c r="K26" s="76"/>
+      <c r="L26" s="76"/>
+      <c r="M26" s="76"/>
+      <c r="N26" s="76"/>
     </row>
     <row r="27" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="59"/>
-      <c r="C27" s="59"/>
-      <c r="D27" s="45" t="s">
+      <c r="B27" s="60"/>
+      <c r="C27" s="60"/>
+      <c r="D27" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="E27" s="45"/>
-      <c r="F27" s="45"/>
-      <c r="G27" s="45"/>
-      <c r="H27" s="45"/>
-      <c r="I27" s="45"/>
-      <c r="J27" s="45"/>
-      <c r="K27" s="45"/>
-      <c r="L27" s="45"/>
-      <c r="M27" s="45"/>
-      <c r="N27" s="45"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="46"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="46"/>
+      <c r="I27" s="46"/>
+      <c r="J27" s="46"/>
+      <c r="K27" s="46"/>
+      <c r="L27" s="46"/>
+      <c r="M27" s="46"/>
+      <c r="N27" s="46"/>
     </row>
     <row r="28" spans="2:14" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="59"/>
-      <c r="C28" s="59"/>
-      <c r="D28" s="75" t="s">
+      <c r="B28" s="60"/>
+      <c r="C28" s="60"/>
+      <c r="D28" s="76" t="s">
         <v>72</v>
       </c>
-      <c r="E28" s="75"/>
-      <c r="F28" s="75"/>
-      <c r="G28" s="75"/>
-      <c r="H28" s="75"/>
-      <c r="I28" s="75"/>
-      <c r="J28" s="75"/>
-      <c r="K28" s="75"/>
-      <c r="L28" s="75"/>
-      <c r="M28" s="75"/>
-      <c r="N28" s="75"/>
+      <c r="E28" s="76"/>
+      <c r="F28" s="76"/>
+      <c r="G28" s="76"/>
+      <c r="H28" s="76"/>
+      <c r="I28" s="76"/>
+      <c r="J28" s="76"/>
+      <c r="K28" s="76"/>
+      <c r="L28" s="76"/>
+      <c r="M28" s="76"/>
+      <c r="N28" s="76"/>
     </row>
     <row r="29" spans="2:14" x14ac:dyDescent="0.35">
       <c r="D29" s="9"/>
@@ -5549,23 +5549,23 @@
       <c r="N29" s="9"/>
     </row>
     <row r="30" spans="2:14" ht="168" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="59" t="s">
+      <c r="B30" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="C30" s="59"/>
-      <c r="D30" s="75" t="s">
+      <c r="C30" s="60"/>
+      <c r="D30" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="E30" s="75"/>
-      <c r="F30" s="75"/>
-      <c r="G30" s="75"/>
-      <c r="H30" s="75"/>
-      <c r="I30" s="75"/>
-      <c r="J30" s="75"/>
-      <c r="K30" s="75"/>
-      <c r="L30" s="75"/>
-      <c r="M30" s="75"/>
-      <c r="N30" s="75"/>
+      <c r="E30" s="76"/>
+      <c r="F30" s="76"/>
+      <c r="G30" s="76"/>
+      <c r="H30" s="76"/>
+      <c r="I30" s="76"/>
+      <c r="J30" s="76"/>
+      <c r="K30" s="76"/>
+      <c r="L30" s="76"/>
+      <c r="M30" s="76"/>
+      <c r="N30" s="76"/>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B31" s="5"/>
@@ -5583,175 +5583,175 @@
       <c r="N31" s="9"/>
     </row>
     <row r="32" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="59" t="s">
+      <c r="B32" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C32" s="59"/>
-      <c r="D32" s="76" t="s">
+      <c r="C32" s="60"/>
+      <c r="D32" s="77" t="s">
         <v>42</v>
       </c>
-      <c r="E32" s="77"/>
-      <c r="F32" s="77"/>
-      <c r="G32" s="77"/>
-      <c r="H32" s="77"/>
-      <c r="I32" s="77"/>
-      <c r="J32" s="77"/>
-      <c r="K32" s="77"/>
-      <c r="L32" s="77"/>
-      <c r="M32" s="77"/>
-      <c r="N32" s="77"/>
+      <c r="E32" s="78"/>
+      <c r="F32" s="78"/>
+      <c r="G32" s="78"/>
+      <c r="H32" s="78"/>
+      <c r="I32" s="78"/>
+      <c r="J32" s="78"/>
+      <c r="K32" s="78"/>
+      <c r="L32" s="78"/>
+      <c r="M32" s="78"/>
+      <c r="N32" s="78"/>
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B33" s="59"/>
-      <c r="C33" s="59"/>
-      <c r="D33" s="77"/>
-      <c r="E33" s="77"/>
-      <c r="F33" s="77"/>
-      <c r="G33" s="77"/>
-      <c r="H33" s="77"/>
-      <c r="I33" s="77"/>
-      <c r="J33" s="77"/>
-      <c r="K33" s="77"/>
-      <c r="L33" s="77"/>
-      <c r="M33" s="77"/>
-      <c r="N33" s="77"/>
+      <c r="B33" s="60"/>
+      <c r="C33" s="60"/>
+      <c r="D33" s="78"/>
+      <c r="E33" s="78"/>
+      <c r="F33" s="78"/>
+      <c r="G33" s="78"/>
+      <c r="H33" s="78"/>
+      <c r="I33" s="78"/>
+      <c r="J33" s="78"/>
+      <c r="K33" s="78"/>
+      <c r="L33" s="78"/>
+      <c r="M33" s="78"/>
+      <c r="N33" s="78"/>
     </row>
     <row r="34" spans="2:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="35" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B35" s="45" t="s">
+      <c r="B35" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="C35" s="45"/>
-      <c r="D35" s="79" t="str">
+      <c r="C35" s="46"/>
+      <c r="D35" s="80" t="str">
         <f>IF($H$9=1,Utileria!$L$15,IF($H$9=2,Utileria!$L$15,IF($H$9=3,Utileria!$L$15,IF($H$9=7,Utileria!L$15,IF($H$9=8,Utileria!$L$15,IF($H$9=16,Utileria!$L$15,IF($H$9=17,Utileria!$L$15,IF($H$9=19,Utileria!$L$15,IF($H$9=24,Utileria!$L$15,IF($H$9=25,Utileria!$L$15,""))))))))))</f>
         <v>¡ATENCIÓN! Para que tu solicitud sea atendida es necesario adjuntar los insumos que a continuación se muestran, en caso de no hacerlo, se puede incurrir en retrasos.</v>
       </c>
-      <c r="E35" s="79"/>
-      <c r="F35" s="79"/>
-      <c r="G35" s="79"/>
-      <c r="H35" s="79"/>
-      <c r="I35" s="79"/>
-      <c r="J35" s="79"/>
-      <c r="K35" s="79"/>
-      <c r="L35" s="79"/>
-      <c r="M35" s="79"/>
-      <c r="N35" s="79"/>
+      <c r="E35" s="80"/>
+      <c r="F35" s="80"/>
+      <c r="G35" s="80"/>
+      <c r="H35" s="80"/>
+      <c r="I35" s="80"/>
+      <c r="J35" s="80"/>
+      <c r="K35" s="80"/>
+      <c r="L35" s="80"/>
+      <c r="M35" s="80"/>
+      <c r="N35" s="80"/>
     </row>
     <row r="36" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D36" s="79"/>
-      <c r="E36" s="79"/>
-      <c r="F36" s="79"/>
-      <c r="G36" s="79"/>
-      <c r="H36" s="79"/>
-      <c r="I36" s="79"/>
-      <c r="J36" s="79"/>
-      <c r="K36" s="79"/>
-      <c r="L36" s="79"/>
-      <c r="M36" s="79"/>
-      <c r="N36" s="79"/>
+      <c r="D36" s="80"/>
+      <c r="E36" s="80"/>
+      <c r="F36" s="80"/>
+      <c r="G36" s="80"/>
+      <c r="H36" s="80"/>
+      <c r="I36" s="80"/>
+      <c r="J36" s="80"/>
+      <c r="K36" s="80"/>
+      <c r="L36" s="80"/>
+      <c r="M36" s="80"/>
+      <c r="N36" s="80"/>
     </row>
     <row r="37" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B37" s="12">
         <f>IF(C37="","", 1)</f>
         <v>1</v>
       </c>
-      <c r="C37" s="57" t="str">
+      <c r="C37" s="58" t="str">
         <f>IF($H$9=1,Utileria!$L$9,IF($H$9=2,Utileria!$L$12,IF($H$9=3,Utileria!$L$11,IF($H$9=7,Utileria!L$6,IF($H$9=8,Utileria!$L$6,IF($H$9=16,Utileria!$L$5,IF($H$9=17,Utileria!$L$4,IF($H$9=19,Utileria!$L$4,IF($H$9=24,Utileria!$L$4,IF($H$9=25,Utileria!$L$4,"N/A"))))))))))</f>
         <v>Ordenes con data de ONIX</v>
       </c>
-      <c r="D37" s="57"/>
-      <c r="E37" s="57"/>
-      <c r="F37" s="57"/>
-      <c r="G37" s="57"/>
-      <c r="H37" s="57"/>
-      <c r="I37" s="57"/>
-      <c r="J37" s="57"/>
-      <c r="K37" s="57"/>
-      <c r="L37" s="57"/>
-      <c r="M37" s="57"/>
-      <c r="N37" s="57"/>
+      <c r="D37" s="58"/>
+      <c r="E37" s="58"/>
+      <c r="F37" s="58"/>
+      <c r="G37" s="58"/>
+      <c r="H37" s="58"/>
+      <c r="I37" s="58"/>
+      <c r="J37" s="58"/>
+      <c r="K37" s="58"/>
+      <c r="L37" s="58"/>
+      <c r="M37" s="58"/>
+      <c r="N37" s="58"/>
     </row>
     <row r="38" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B38" s="12" t="str">
         <f>IF(C38="","", 2)</f>
         <v/>
       </c>
-      <c r="C38" s="57" t="str">
+      <c r="C38" s="58" t="str">
         <f>IF($H$9=1,Utileria!$L$10,IF($H$9=7,Utileria!$L$8,IF($H$9=8,Utileria!$L$7,IF($H$9=2,Utileria!$L$13,""))))</f>
         <v/>
       </c>
-      <c r="D38" s="57"/>
-      <c r="E38" s="57"/>
-      <c r="F38" s="57"/>
-      <c r="G38" s="57"/>
-      <c r="H38" s="57"/>
-      <c r="I38" s="57"/>
-      <c r="J38" s="57"/>
-      <c r="K38" s="57"/>
-      <c r="L38" s="57"/>
-      <c r="M38" s="57"/>
-      <c r="N38" s="57"/>
+      <c r="D38" s="58"/>
+      <c r="E38" s="58"/>
+      <c r="F38" s="58"/>
+      <c r="G38" s="58"/>
+      <c r="H38" s="58"/>
+      <c r="I38" s="58"/>
+      <c r="J38" s="58"/>
+      <c r="K38" s="58"/>
+      <c r="L38" s="58"/>
+      <c r="M38" s="58"/>
+      <c r="N38" s="58"/>
     </row>
     <row r="39" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="40" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B40" s="45" t="s">
+      <c r="B40" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="C40" s="45"/>
-      <c r="D40" s="45"/>
-      <c r="E40" s="45"/>
-      <c r="F40" s="45"/>
-      <c r="G40" s="45"/>
-      <c r="H40" s="45"/>
-      <c r="I40" s="45"/>
-      <c r="J40" s="45"/>
-      <c r="K40" s="45"/>
-      <c r="L40" s="45"/>
-      <c r="M40" s="45"/>
-      <c r="N40" s="45"/>
+      <c r="C40" s="46"/>
+      <c r="D40" s="46"/>
+      <c r="E40" s="46"/>
+      <c r="F40" s="46"/>
+      <c r="G40" s="46"/>
+      <c r="H40" s="46"/>
+      <c r="I40" s="46"/>
+      <c r="J40" s="46"/>
+      <c r="K40" s="46"/>
+      <c r="L40" s="46"/>
+      <c r="M40" s="46"/>
+      <c r="N40" s="46"/>
     </row>
     <row r="41" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="42" spans="2:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B42" s="46" t="s">
+      <c r="B42" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C42" s="46"/>
-      <c r="D42" s="74" t="s">
+      <c r="C42" s="47"/>
+      <c r="D42" s="75" t="s">
         <v>36</v>
       </c>
-      <c r="E42" s="74"/>
-      <c r="F42" s="74"/>
-      <c r="G42" s="74"/>
-      <c r="H42" s="45" t="s">
+      <c r="E42" s="75"/>
+      <c r="F42" s="75"/>
+      <c r="G42" s="75"/>
+      <c r="H42" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="I42" s="45"/>
-      <c r="J42" s="74" t="s">
+      <c r="I42" s="46"/>
+      <c r="J42" s="75" t="s">
         <v>66</v>
       </c>
-      <c r="K42" s="74"/>
-      <c r="L42" s="74"/>
-      <c r="M42" s="74"/>
+      <c r="K42" s="75"/>
+      <c r="L42" s="75"/>
+      <c r="M42" s="75"/>
     </row>
     <row r="43" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="44" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B44" s="45" t="s">
+      <c r="B44" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="C44" s="45"/>
-      <c r="D44" s="78" t="s">
+      <c r="C44" s="46"/>
+      <c r="D44" s="79" t="s">
         <v>44</v>
       </c>
-      <c r="E44" s="78"/>
-      <c r="F44" s="78"/>
-      <c r="G44" s="78"/>
-      <c r="H44" s="78"/>
-      <c r="I44" s="78"/>
-      <c r="J44" s="78"/>
-      <c r="K44" s="78"/>
-      <c r="L44" s="78"/>
-      <c r="M44" s="78"/>
-      <c r="N44" s="78"/>
+      <c r="E44" s="79"/>
+      <c r="F44" s="79"/>
+      <c r="G44" s="79"/>
+      <c r="H44" s="79"/>
+      <c r="I44" s="79"/>
+      <c r="J44" s="79"/>
+      <c r="K44" s="79"/>
+      <c r="L44" s="79"/>
+      <c r="M44" s="79"/>
+      <c r="N44" s="79"/>
     </row>
     <row r="45" spans="2:14" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B45" s="11"/>
@@ -6726,7 +6726,7 @@
       <c r="C33">
         <v>28</v>
       </c>
-      <c r="D33" s="80" t="s">
+      <c r="D33" s="43" t="s">
         <v>142</v>
       </c>
       <c r="E33" s="1"/>

</xml_diff>